<commit_message>
PCB: C27 to 0603 10uF (keep nominal, full 10V margin)
Per request, C27 (STO local bulk) moves from the interim 4.7uF 10V 0402 back to
10uF at 10V by going 0603 (GRM188R61A106KE69D), matching C25's approach and now
sharing the C4/C13 reel. Keeps the 10uF nominal with full voltage margin at the
4.65V STO node; land grows from 0402 (traces reworked on the board). Synced across
schematic, both BOMs, and the docs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PBK3zFENdvoGtn8yP7qPA8
</commit_message>
<xml_diff>
--- a/PCB/solar-glow-drh-v4_0-BOM-assembly.xlsx
+++ b/PCB/solar-glow-drh-v4_0-BOM-assembly.xlsx
@@ -2150,12 +2150,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>4.7 µF, 10 V, 0402, X5R</t>
+          <t>10 µF, 10 V, 0603, X5R</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2165,22 +2165,22 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>GRM155R61A475MEAAD</t>
+          <t>GRM188R61A106KE69D</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>v4 NEW</t>
+          <t>LAND REWORK</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Bumped 6.3V 10uF -&gt; 10V 4.7uF: STO rides to 4.65V where a 6.3V 0402 is thin (74% of rating) and heavily derated. 10V is the point; HF role (the 1F tank is the bulk). Reuses the 4.7uF 10V 0402 part.</t>
+          <t>Moved to 0603 to keep 10uF at 10V (per request; matches C25's approach). STO rides to 4.65V where a 6.3V 0402 was thin + heavily derated; 10V 0603 gives full margin and effective bulk. Shares the C4/C13 10uF 10V 0603 reel. Land grows from 0402 - PCB rework.</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>GRM155R61A475MEAAD-ND (format-derived - confirm at cart)</t>
+          <t>GRM188R61A106KE69D-ND (format-derived - confirm at cart)</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,6 @@
         <v/>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
PCB: fix L2 schematic footprint to the 2520 land (was still 0603)
Review of the uploaded copper caught L2: the four caps (C4/C13/C27 -> 0603,
C23 -> 2.2uF) came through correctly, but L2 was still on a 0603 land. Root
cause: L2's schematic Footprint field was left at Inductor_SMD:L_0603_1608Metric
(the land-growth was only noted in the description/BOM), so Update-PCB had nothing
to change and silently kept the 0603 land -- and the DFE252010F-100M is 2.5x2.0 mm.

Fix: set L2's footprint to the KiCad stock Inductor_SMD:L_1008_2520Metric (pads
1.25x2.2 mm at +/-1.075 mm), the generic land for the 2.5x2.0 mm (1008/2520)
package. Verified the footprint exists in the current KiCad library. Synced the
L2 rows in both BOMs and the docs. Next: re-run Update-PCB to place the 2520 land,
then route L2.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PBK3zFENdvoGtn8yP7qPA8
</commit_message>
<xml_diff>
--- a/PCB/solar-glow-drh-v4_0-BOM-assembly.xlsx
+++ b/PCB/solar-glow-drh-v4_0-BOM-assembly.xlsx
@@ -1809,7 +1809,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>2.5x2.0x1.0 mm (DFE252010); land grows past 0603</t>
+          <t>1008/2520 (L_1008_2520Metric), 2.5x2.0 mm</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1824,12 +1824,12 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>v4 NEW - LAND REWORK</t>
+          <t>v4 - ROUTE L2</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>AEM10300 datasheet Table 11 LDCDC = DFE252010F-100M (10 uH, 1.76 A, &gt;=1 A / &gt;=10 MHz). Land grows past 0603 - PCB rework pending.</t>
+          <t>Murata DFE252010F-100M (10uH, 1.76A) per aem10300.pdf Table 11 / 9.8.2 (&gt;=1A, &gt;=10MHz, low ESR). Schematic footprint set to the KiCad stock 1008/2520 land (Inductor_SMD:L_1008_2520Metric, pads 1.25x2.2mm), the generic land for the 2.5x2.0mm package. Re-run Update-PCB to place it, then route (the earlier upload still had L2 on a 0603 land). Swap to Murata's exact DFE252010F land later if preferred.</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">

</xml_diff>